<commit_message>
验收 b02：UnitySkills Play Mode 走查通过，任务表 P0-001~P0-008 置为已完成
- tasks.md：5 项 Play Mode 走查（2.7/3.6/3.8/4.4/5.6）勾选完成
- verification.md：补充 Editor 内实测验收证据与判定
- 任务表：P0-001~P0-008 状态置「已完成」并备注批次
- 分批执行计划：b01/b02 标记已完成，b03 为下一批
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -462,9 +462,6 @@
           <t>第一版开发任务表使用说明</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -886,11 +883,15 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>b01 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -966,11 +967,15 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>b01 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1046,11 +1051,15 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>b01 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1126,11 +1135,15 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>b01 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1206,11 +1219,15 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>b02 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1286,11 +1303,15 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>b02 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1366,11 +1387,15 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>b02 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1446,11 +1471,15 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>b02 完成并通过验收</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -11074,8 +11103,6 @@
           <t>约73~73</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
验收 b03：UnitySkills Play Mode 走查通过，任务表 P0-009~P0-012 置为已完成
- 探针 15 项断言全通过：存档往返/独立/损坏/版本拒绝、随机同种子/计数/重置、演算日志开关/重放、诊断场景

- 静态检查：verify_project_assemblies.py 通过（Board 零引擎）、audit_framework_purity.py 通过、编译零错误

- 任务表 P0-009~P0-012 状态置为已完成；verification.md 记录证据；分批计划推进至 b04
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -1555,11 +1555,15 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>b03 完成并通过验收（存档/随机/配置字段/诊断）</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1635,11 +1639,15 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>b03 完成并通过验收（存档/随机/配置字段/诊断）</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1715,11 +1723,15 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>b03 完成并通过验收（存档/随机/配置字段/诊断）</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1795,11 +1807,15 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>b03 完成并通过验收（存档/随机/配置字段/诊断）</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
验收 b05：UnitySkills Play Mode 走查通过（69/69），任务表 P1-001/P1-002 置为已完成
蜂窝格各 n 档位生成、坐标方向换算、每格单实体占用与固定设施锁盘面移动限制全部通过；Board 层零引擎依赖，纯度审计与程序集校验通过。
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -1975,11 +1975,15 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>蜂窝格棋盘数据模型（轴向坐标/六方向/边长n分档/合法格/分层）完成，Play Mode 验收 69/69 通过</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2055,11 +2059,15 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>棋子实体与占用层（零件/设施/任务标记/待维修对象基类，每格单实体，固定设施锁盘面）完成，Play Mode 验收 69/69 通过</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
验收 b09：任务表 P1-010/P1-011/P1-012/P1-013 置已完成 + 验证记录
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -2731,11 +2731,15 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>b09 验收通过(31/31)：机械臂+轮关/过轮判定+种子复现+第一步预演</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2811,11 +2815,15 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>b09 验收通过(31/31)：机械臂+轮关/过轮判定+种子复现+第一步预演</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2891,11 +2899,15 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>b09 验收通过(31/31)：机械臂+轮关/过轮判定+种子复现+第一步预演</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2971,11 +2983,15 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>b09 验收通过(31/31)：机械臂+轮关/过轮判定+种子复现+第一步预演</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">

</xml_diff>

<commit_message>
验收 b10：任务表 P1-014/P1-015/P1-016/P1-017 置已完成 + 验证记录
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -3067,11 +3067,15 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>b10 验收通过(31/31)：盘面视图+棋子/设施/标记表现+操作循环UI+六分区HUD</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3147,11 +3151,15 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>b10 验收通过(31/31)：盘面视图+棋子/设施/标记表现+操作循环UI+六分区HUD</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3227,11 +3235,15 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>b10 验收通过(31/31)：盘面视图+棋子/设施/标记表现+操作循环UI+六分区HUD</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3307,11 +3319,15 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>b10 验收通过(31/31)：盘面视图+棋子/设施/标记表现+操作循环UI+六分区HUD</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">

</xml_diff>

<commit_message>
验收 b11：任务表 P1-018/P1-019/P1-020/P1-021 置已完成 + 验证记录
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -3403,11 +3403,15 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>b11 验收通过(25/25)：四选一框架+Buff数据结构与首批20项+暂停撤退菜单+关卡盘面配置表</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3483,11 +3487,15 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>b11 验收通过(25/25)：四选一框架+Buff数据结构与首批20项+暂停撤退菜单+关卡盘面配置表</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3563,11 +3571,15 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>b11 验收通过(25/25)：四选一框架+Buff数据结构与首批20项+暂停撤退菜单+关卡盘面配置表</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3643,11 +3655,15 @@
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>b11 验收通过(25/25)：四选一框架+Buff数据结构与首批20项+暂停撤退菜单+关卡盘面配置表</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">

</xml_diff>

<commit_message>
b38 完成：构建与 G6 门（P6-009~P6-012）
BuildConfig 构建口径 + VersionConfig 版本/渠道口径 + ReleaseCoverageService 投放覆盖审计 + G6 门集成探针 6/6 通过（新档自走完整链路），G6 第一版完成里程碑关闭；任务表 P6-009~012 置「已完成」。
</commit_message>
<xml_diff>
--- a/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
+++ b/Docs/GameDesign/10-开发计划/第一版开发任务表.xlsx
@@ -9699,7 +9699,7 @@
       </c>
       <c r="P110" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q110" s="2" t="inlineStr"/>
@@ -9779,7 +9779,7 @@
       </c>
       <c r="P111" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q111" s="2" t="inlineStr"/>
@@ -9859,7 +9859,7 @@
       </c>
       <c r="P112" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q112" s="2" t="inlineStr"/>
@@ -9939,7 +9939,7 @@
       </c>
       <c r="P113" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="Q113" s="2" t="inlineStr"/>

</xml_diff>